<commit_message>
Implement Tab1 sales plan vs actual dashboard (FastAPI + React)
- FastAPI backend serving sample JSON data with static frontend hosting
- React (Vite) frontend: KPI cards, 5-stage pipeline with click filter,
  monthly plan-vs-actual combo chart (won/revenue and monthly/cumulative
  toggles), BU x channel achievement heatmap, sortable/searchable
  opportunity table with slide-in detail panel; Tab2 placeholder
- Rescale sample data for coherence: annual plan 6.4B KRW, add 9 H1
  won/revenue deals (80% overall achievement), regenerate Excel files
- DESIGN.md rewritten in canonical format from the built system, with
  .impeccable/design.json sidecar; chart palette CVD-validated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S8p4s3WR2VZ9gm23wpN3hc
</commit_message>
<xml_diff>
--- a/excel/sales_pipeline_template.xlsx
+++ b/excel/sales_pipeline_template.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:W25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2108,6 +2108,849 @@
       <c r="W16" s="2" t="inlineStr">
         <is>
           <t>교육청 개별 입찰공고 센싱 기반</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>A제조 본사·사무동 복합기 MPS 구축</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>A제조(반도체 후공정)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>직판</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>B2B기업</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>복합기·MPS</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>WF-C879R</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>740000000</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>매출 인식</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>부서별 개별 프린터 난립, 출력비용 관리 불가</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>보안출력·관제 SW 포함 5년 계약</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>김민준 차장</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>1분기 납품·검수 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>F대학병원 병동 복합기 MPS 5년 계약</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>F대학병원</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>총판</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Q오피스솔루션</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>B2B기업</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>복합기·MPS</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>AM-C400</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>920000000</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>매출 인식</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>병동별 노후 장비 혼재, 유지비 급증</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>의료정보 보안출력 필수, 24시간 A/S</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>김민준 차장</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>2월 계약·상반기 매출 인식 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>경기OO교육청 중학교 전자교탁 프로젝터 240대</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>경기OO교육청</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>PJT</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>직판</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>B2G공공</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>교육용 프로젝터</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>EB-770F</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>680000000</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>매출 인식</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>중학교 전자교탁 사업 1차분 발주</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>초단초점, 전자펜 인터랙티브</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>박지훈 과장</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>4월 낙찰·납품 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>OO시청 시민홀 대형 레이저 프로젝터</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>OO시청</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>PJT</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>총판</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Q오피스솔루션</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>B2G공공</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>비즈니스 프로젝터</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>EB-PU2220B</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>660000000</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>계약 완료(수주)</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>시민홀 리모델링에 따른 대형 영상장비 신설</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>20,000루멘, WUXGA, 스택 투사</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>박지훈 과장</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>5월 수주, 3분기 설치 예정</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>C전자부품 SCARA 1차 라인 증설 확정분</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>C전자부품</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>RBT</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>직판</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>B2B기업</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>SCARA 로봇</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>GX4-B351S</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>590000000</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>계약 완료(수주)</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>1차 도입 라인 성과 확인 후 확정 발주</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>기존 6대와 동일 사양·통합 제어</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0005</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>최유진 차장</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>6월 수주, 4분기 설치</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>D디스플레이 헤드모듈 상반기 정기 공급</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>D디스플레이</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>직판</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>B2B기업</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>잉크젯 헤드(부품)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>PrecisionCore 헤드모듈</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>560000000</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>매출 인식</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>기존 라인 소모성 헤드모듈 정기 교체 수요</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>기존 QUAL 통과 사양 동일</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>정현우 부장</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>연간 공급계약 상반기분 인식</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>E물류 1·2센터 라벨프린터 교체</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>E물류</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>총판</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>P총판상사</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>B2B기업</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>컬러 라벨프린터</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>CW-C6500</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>계약 완료(수주)</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>기존 장비 노후로 인쇄 품질 저하</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>WMS 연동 유지</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>이서연 대리</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>6월 수주, 순차 교체 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>C전자부품 협력사 GX4 로봇 2대</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>C전자부품</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>RBT</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>총판</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>P총판상사</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>B2B기업</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>SCARA 로봇</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>GX4-B351S</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>매출 인식</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>협력사 소형 조립 셀 자동화</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>표준 사양</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>최유진 차장</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>협력사 소개 건, 납품 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>A제조 후공정 잉크젯 1차 도입분</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>A제조(반도체 후공정)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>직판</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>B2B기업</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>산업용 잉크젯</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>WF-C21000</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>520000000</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>계약 완료(수주)</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>증설 라인 가동 전 선행 도입 물량</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>본계약과 동일 사양</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>OPP-2026-0001</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>기존고객</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>김민준 차장</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>증설 본건(OPP-2026-0001)의 선행 발주분</t>
         </is>
       </c>
     </row>
@@ -2194,7 +3037,7 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>350000000</v>
+        <v>70000000</v>
       </c>
     </row>
     <row r="3">
@@ -2215,7 +3058,7 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>350000000</v>
+        <v>70000000</v>
       </c>
     </row>
     <row r="4">
@@ -2236,7 +3079,7 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>450000000</v>
+        <v>90000000</v>
       </c>
     </row>
     <row r="5">
@@ -2257,7 +3100,7 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>450000000</v>
+        <v>90000000</v>
       </c>
     </row>
     <row r="6">
@@ -2278,7 +3121,7 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>500000000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="7">
@@ -2299,7 +3142,7 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>550000000</v>
+        <v>110000000</v>
       </c>
     </row>
     <row r="8">
@@ -2320,7 +3163,7 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>500000000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="9">
@@ -2341,7 +3184,7 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>500000000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="10">
@@ -2362,7 +3205,7 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>600000000</v>
+        <v>120000000</v>
       </c>
     </row>
     <row r="11">
@@ -2383,7 +3226,7 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>600000000</v>
+        <v>120000000</v>
       </c>
     </row>
     <row r="12">
@@ -2404,7 +3247,7 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>600000000</v>
+        <v>120000000</v>
       </c>
     </row>
     <row r="13">
@@ -2425,7 +3268,7 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>550000000</v>
+        <v>110000000</v>
       </c>
     </row>
     <row r="14">
@@ -2446,7 +3289,7 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>408000000</v>
+        <v>82000000</v>
       </c>
     </row>
     <row r="15">
@@ -2467,7 +3310,7 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>408000000</v>
+        <v>82000000</v>
       </c>
     </row>
     <row r="16">
@@ -2488,7 +3331,7 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>525000000</v>
+        <v>105000000</v>
       </c>
     </row>
     <row r="17">
@@ -2509,7 +3352,7 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>525000000</v>
+        <v>105000000</v>
       </c>
     </row>
     <row r="18">
@@ -2530,7 +3373,7 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>583000000</v>
+        <v>117000000</v>
       </c>
     </row>
     <row r="19">
@@ -2551,7 +3394,7 @@
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>642000000</v>
+        <v>128000000</v>
       </c>
     </row>
     <row r="20">
@@ -2572,7 +3415,7 @@
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>583000000</v>
+        <v>117000000</v>
       </c>
     </row>
     <row r="21">
@@ -2593,7 +3436,7 @@
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>583000000</v>
+        <v>117000000</v>
       </c>
     </row>
     <row r="22">
@@ -2614,7 +3457,7 @@
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>700000000</v>
+        <v>140000000</v>
       </c>
     </row>
     <row r="23">
@@ -2635,7 +3478,7 @@
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>700000000</v>
+        <v>140000000</v>
       </c>
     </row>
     <row r="24">
@@ -2656,7 +3499,7 @@
         </is>
       </c>
       <c r="E24" s="3" t="n">
-        <v>700000000</v>
+        <v>140000000</v>
       </c>
     </row>
     <row r="25">
@@ -2677,7 +3520,7 @@
         </is>
       </c>
       <c r="E25" s="3" t="n">
-        <v>643000000</v>
+        <v>127000000</v>
       </c>
     </row>
     <row r="26">
@@ -2698,7 +3541,7 @@
         </is>
       </c>
       <c r="E26" s="3" t="n">
-        <v>262000000</v>
+        <v>52000000</v>
       </c>
     </row>
     <row r="27">
@@ -2719,7 +3562,7 @@
         </is>
       </c>
       <c r="E27" s="3" t="n">
-        <v>262000000</v>
+        <v>52000000</v>
       </c>
     </row>
     <row r="28">
@@ -2740,7 +3583,7 @@
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>338000000</v>
+        <v>68000000</v>
       </c>
     </row>
     <row r="29">
@@ -2761,7 +3604,7 @@
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>338000000</v>
+        <v>68000000</v>
       </c>
     </row>
     <row r="30">
@@ -2782,7 +3625,7 @@
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>375000000</v>
+        <v>75000000</v>
       </c>
     </row>
     <row r="31">
@@ -2803,7 +3646,7 @@
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>412000000</v>
+        <v>83000000</v>
       </c>
     </row>
     <row r="32">
@@ -2824,7 +3667,7 @@
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>375000000</v>
+        <v>75000000</v>
       </c>
     </row>
     <row r="33">
@@ -2845,7 +3688,7 @@
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>375000000</v>
+        <v>75000000</v>
       </c>
     </row>
     <row r="34">
@@ -2866,7 +3709,7 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>450000000</v>
+        <v>90000000</v>
       </c>
     </row>
     <row r="35">
@@ -2887,7 +3730,7 @@
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>450000000</v>
+        <v>90000000</v>
       </c>
     </row>
     <row r="36">
@@ -2908,7 +3751,7 @@
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>450000000</v>
+        <v>90000000</v>
       </c>
     </row>
     <row r="37">
@@ -2929,7 +3772,7 @@
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>413000000</v>
+        <v>82000000</v>
       </c>
     </row>
     <row r="38">
@@ -2950,7 +3793,7 @@
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>204000000</v>
+        <v>41000000</v>
       </c>
     </row>
     <row r="39">
@@ -2971,7 +3814,7 @@
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>204000000</v>
+        <v>41000000</v>
       </c>
     </row>
     <row r="40">
@@ -2992,7 +3835,7 @@
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>262000000</v>
+        <v>52000000</v>
       </c>
     </row>
     <row r="41">
@@ -3013,7 +3856,7 @@
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>262000000</v>
+        <v>52000000</v>
       </c>
     </row>
     <row r="42">
@@ -3034,7 +3877,7 @@
         </is>
       </c>
       <c r="E42" s="3" t="n">
-        <v>292000000</v>
+        <v>58000000</v>
       </c>
     </row>
     <row r="43">
@@ -3055,7 +3898,7 @@
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>321000000</v>
+        <v>64000000</v>
       </c>
     </row>
     <row r="44">
@@ -3076,7 +3919,7 @@
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>292000000</v>
+        <v>58000000</v>
       </c>
     </row>
     <row r="45">
@@ -3097,7 +3940,7 @@
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>292000000</v>
+        <v>58000000</v>
       </c>
     </row>
     <row r="46">
@@ -3118,7 +3961,7 @@
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>350000000</v>
+        <v>70000000</v>
       </c>
     </row>
     <row r="47">
@@ -3139,7 +3982,7 @@
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>350000000</v>
+        <v>70000000</v>
       </c>
     </row>
     <row r="48">
@@ -3160,7 +4003,7 @@
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>350000000</v>
+        <v>70000000</v>
       </c>
     </row>
     <row r="49">
@@ -3181,7 +4024,7 @@
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>321000000</v>
+        <v>66000000</v>
       </c>
     </row>
     <row r="50">
@@ -3202,7 +4045,7 @@
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>321000000</v>
+        <v>64000000</v>
       </c>
     </row>
     <row r="51">
@@ -3223,7 +4066,7 @@
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>321000000</v>
+        <v>64000000</v>
       </c>
     </row>
     <row r="52">
@@ -3244,7 +4087,7 @@
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>412000000</v>
+        <v>82000000</v>
       </c>
     </row>
     <row r="53">
@@ -3265,7 +4108,7 @@
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>412000000</v>
+        <v>82000000</v>
       </c>
     </row>
     <row r="54">
@@ -3286,7 +4129,7 @@
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>458000000</v>
+        <v>92000000</v>
       </c>
     </row>
     <row r="55">
@@ -3307,7 +4150,7 @@
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>504000000</v>
+        <v>101000000</v>
       </c>
     </row>
     <row r="56">
@@ -3328,7 +4171,7 @@
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>458000000</v>
+        <v>92000000</v>
       </c>
     </row>
     <row r="57">
@@ -3349,7 +4192,7 @@
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>458000000</v>
+        <v>92000000</v>
       </c>
     </row>
     <row r="58">
@@ -3370,7 +4213,7 @@
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>550000000</v>
+        <v>110000000</v>
       </c>
     </row>
     <row r="59">
@@ -3391,7 +4234,7 @@
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>550000000</v>
+        <v>110000000</v>
       </c>
     </row>
     <row r="60">
@@ -3412,7 +4255,7 @@
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>550000000</v>
+        <v>110000000</v>
       </c>
     </row>
     <row r="61">
@@ -3433,7 +4276,7 @@
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>506000000</v>
+        <v>101000000</v>
       </c>
     </row>
     <row r="62">
@@ -3454,7 +4297,7 @@
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>58000000</v>
+        <v>12000000</v>
       </c>
     </row>
     <row r="63">
@@ -3475,7 +4318,7 @@
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>58000000</v>
+        <v>12000000</v>
       </c>
     </row>
     <row r="64">
@@ -3496,7 +4339,7 @@
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>75000000</v>
+        <v>15000000</v>
       </c>
     </row>
     <row r="65">
@@ -3517,7 +4360,7 @@
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>75000000</v>
+        <v>15000000</v>
       </c>
     </row>
     <row r="66">
@@ -3538,7 +4381,7 @@
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>83000000</v>
+        <v>17000000</v>
       </c>
     </row>
     <row r="67">
@@ -3559,7 +4402,7 @@
         </is>
       </c>
       <c r="E67" s="3" t="n">
-        <v>92000000</v>
+        <v>18000000</v>
       </c>
     </row>
     <row r="68">
@@ -3580,7 +4423,7 @@
         </is>
       </c>
       <c r="E68" s="3" t="n">
-        <v>83000000</v>
+        <v>17000000</v>
       </c>
     </row>
     <row r="69">
@@ -3601,7 +4444,7 @@
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>83000000</v>
+        <v>17000000</v>
       </c>
     </row>
     <row r="70">
@@ -3622,7 +4465,7 @@
         </is>
       </c>
       <c r="E70" s="3" t="n">
-        <v>100000000</v>
+        <v>20000000</v>
       </c>
     </row>
     <row r="71">
@@ -3643,7 +4486,7 @@
         </is>
       </c>
       <c r="E71" s="3" t="n">
-        <v>100000000</v>
+        <v>20000000</v>
       </c>
     </row>
     <row r="72">
@@ -3664,7 +4507,7 @@
         </is>
       </c>
       <c r="E72" s="3" t="n">
-        <v>100000000</v>
+        <v>20000000</v>
       </c>
     </row>
     <row r="73">
@@ -3685,7 +4528,7 @@
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>93000000</v>
+        <v>17000000</v>
       </c>
     </row>
     <row r="74">
@@ -3706,7 +4549,7 @@
         </is>
       </c>
       <c r="E74" s="3" t="n">
-        <v>233000000</v>
+        <v>47000000</v>
       </c>
     </row>
     <row r="75">
@@ -3727,7 +4570,7 @@
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>233000000</v>
+        <v>47000000</v>
       </c>
     </row>
     <row r="76">
@@ -3748,7 +4591,7 @@
         </is>
       </c>
       <c r="E76" s="3" t="n">
-        <v>300000000</v>
+        <v>60000000</v>
       </c>
     </row>
     <row r="77">
@@ -3769,7 +4612,7 @@
         </is>
       </c>
       <c r="E77" s="3" t="n">
-        <v>300000000</v>
+        <v>60000000</v>
       </c>
     </row>
     <row r="78">
@@ -3790,7 +4633,7 @@
         </is>
       </c>
       <c r="E78" s="3" t="n">
-        <v>333000000</v>
+        <v>67000000</v>
       </c>
     </row>
     <row r="79">
@@ -3811,7 +4654,7 @@
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>367000000</v>
+        <v>73000000</v>
       </c>
     </row>
     <row r="80">
@@ -3832,7 +4675,7 @@
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>333000000</v>
+        <v>67000000</v>
       </c>
     </row>
     <row r="81">
@@ -3853,7 +4696,7 @@
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>333000000</v>
+        <v>67000000</v>
       </c>
     </row>
     <row r="82">
@@ -3874,7 +4717,7 @@
         </is>
       </c>
       <c r="E82" s="3" t="n">
-        <v>400000000</v>
+        <v>80000000</v>
       </c>
     </row>
     <row r="83">
@@ -3895,7 +4738,7 @@
         </is>
       </c>
       <c r="E83" s="3" t="n">
-        <v>400000000</v>
+        <v>80000000</v>
       </c>
     </row>
     <row r="84">
@@ -3916,7 +4759,7 @@
         </is>
       </c>
       <c r="E84" s="3" t="n">
-        <v>400000000</v>
+        <v>80000000</v>
       </c>
     </row>
     <row r="85">
@@ -3937,7 +4780,7 @@
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>368000000</v>
+        <v>72000000</v>
       </c>
     </row>
     <row r="86">
@@ -3958,7 +4801,7 @@
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>29000000</v>
+        <v>6000000</v>
       </c>
     </row>
     <row r="87">
@@ -3979,7 +4822,7 @@
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>29000000</v>
+        <v>6000000</v>
       </c>
     </row>
     <row r="88">
@@ -4000,7 +4843,7 @@
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>38000000</v>
+        <v>8000000</v>
       </c>
     </row>
     <row r="89">
@@ -4021,7 +4864,7 @@
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>38000000</v>
+        <v>8000000</v>
       </c>
     </row>
     <row r="90">
@@ -4042,7 +4885,7 @@
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>42000000</v>
+        <v>8000000</v>
       </c>
     </row>
     <row r="91">
@@ -4063,7 +4906,7 @@
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>46000000</v>
+        <v>9000000</v>
       </c>
     </row>
     <row r="92">
@@ -4084,7 +4927,7 @@
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>42000000</v>
+        <v>8000000</v>
       </c>
     </row>
     <row r="93">
@@ -4105,7 +4948,7 @@
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>42000000</v>
+        <v>8000000</v>
       </c>
     </row>
     <row r="94">
@@ -4126,7 +4969,7 @@
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>50000000</v>
+        <v>10000000</v>
       </c>
     </row>
     <row r="95">
@@ -4147,7 +4990,7 @@
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>50000000</v>
+        <v>10000000</v>
       </c>
     </row>
     <row r="96">
@@ -4168,7 +5011,7 @@
         </is>
       </c>
       <c r="E96" s="3" t="n">
-        <v>50000000</v>
+        <v>10000000</v>
       </c>
     </row>
     <row r="97">
@@ -4189,7 +5032,7 @@
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>44000000</v>
+        <v>9000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>